<commit_message>
feat: complete in-game encyclopedia
complete in-game encyclopedia (Teaching.pck), special lessons
(Lesson.pck), and UI tooltips
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/ui_strings.xlsx
+++ b/mod_project/data_tables/ui_strings.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -555,6 +555,106 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>StringData_0256.bin</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>256</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Check the Libra Book.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Check the Libra Book (9 seals unlock monster stats/HP in scan).</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>StringData_0458.bin</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>458</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Enchant your equipment.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Forge equipment (+1 to +9) to inherit Sealbook primary enchants.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>StringData_0528.bin</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>528</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Create Sealbooks using captured monsters.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Create Sealbooks (9 monsters) to unlock combat scan &amp; forge enchants.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>StringData_0529.bin</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>529</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Create Grand Sealbooks using captured mutants.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Create Grand Sealbooks (1 mutant) for party auras &amp; monster summons.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: implement combat command tooltips
implement combat command tooltips, dungeon trap lethality, trophy
milestones, and attendant advisory dialogue
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/ui_strings.xlsx
+++ b/mod_project/data_tables/ui_strings.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,7 +521,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Party skills increase in efficacy based on the number of awards earned.</t>
+          <t>Party skills gain +1% power per 5 awards earned (up to 50 awards).</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -650,6 +650,156 @@
         </is>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>StringData_0199.bin</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>199</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Use a skill in which team members join forces.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Execute combo using consecutive turns. Consumes 10-25% Max TP &amp; Pep.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>StringData_0200.bin</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>200</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Attack with your equipped weapon.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Basic attack. Range penalty (-50% dmg) applies beyond weapon reach.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>StringData_0201.bin</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>201</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Strike using techniques or spells.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Techniques strike instantly. Spells require chant and can be interrupted.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>StringData_0202.bin</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>202</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Take a defensive stance to guard against enemy attacks.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Halve damage (50%), cut delay to 0.67x, &amp; prevent crits and interrupts.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>StringData_0203.bin</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>203</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Utilize an item in your possession.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Use consumable item. Recovery is fixed and unaffected by user stats.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>StringData_0204.bin</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>204</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Attempt to escape from battle.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Flee battle (AGI check). Boss and mutant encounters cannot be fled.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>

</xml_diff>